<commit_message>
update export tool to fit the template
</commit_message>
<xml_diff>
--- a/results/result1.xlsx
+++ b/results/result1.xlsx
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>1406.329866666666</v>
+        <v>1406.3299</v>
       </c>
     </row>
     <row r="4" ht="14" customHeight="1">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>1407.38385</v>
+        <v>1407.3839</v>
       </c>
     </row>
     <row r="5" ht="14" customHeight="1">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>1409.07395</v>
+        <v>1409.074</v>
       </c>
     </row>
     <row r="6" ht="14" customHeight="1">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>1409.80455</v>
+        <v>1409.8046</v>
       </c>
     </row>
     <row r="7" ht="14" customHeight="1">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>576.6400166666666</v>
+        <v>576.64</v>
       </c>
     </row>
     <row r="8" ht="14" customHeight="1">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>577.9938666666667</v>
+        <v>577.9939000000001</v>
       </c>
     </row>
     <row r="10" ht="14" customHeight="1">
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>911.1613833333333</v>
+        <v>911.1614</v>
       </c>
     </row>
     <row r="11" ht="14" customHeight="1">
@@ -564,7 +564,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>580.41545</v>
+        <v>580.4154</v>
       </c>
     </row>
     <row r="12" ht="14" customHeight="1">
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>582.5140166666666</v>
+        <v>582.514</v>
       </c>
     </row>
     <row r="13" ht="14" customHeight="1">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>583.0740499999999</v>
+        <v>583.074</v>
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>584.2049166666666</v>
+        <v>584.2049</v>
       </c>
     </row>
     <row r="15" ht="14" customHeight="1">
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>585.4397833333333</v>
+        <v>585.4398</v>
       </c>
     </row>
     <row r="16" ht="14" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>586.1447499999999</v>
+        <v>586.1446999999999</v>
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>586.3207666666666</v>
+        <v>586.3208</v>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>587.8210166666667</v>
+        <v>587.821</v>
       </c>
     </row>
     <row r="21" ht="14" customHeight="1">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>589.5475666666666</v>
+        <v>589.5476</v>
       </c>
     </row>
     <row r="22" ht="14" customHeight="1">
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>590.8134666666666</v>
+        <v>590.8135</v>
       </c>
     </row>
     <row r="23" ht="14" customHeight="1">
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>590.2131166666666</v>
+        <v>590.2131000000001</v>
       </c>
     </row>
     <row r="24" ht="14" customHeight="1">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>591.0662666666666</v>
+        <v>591.0663</v>
       </c>
     </row>
     <row r="25" ht="14" customHeight="1">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>593.3678333333332</v>
+        <v>593.3678</v>
       </c>
     </row>
     <row r="26" ht="14" customHeight="1">
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>593.6596833333333</v>
+        <v>593.6597</v>
       </c>
     </row>
     <row r="27" ht="14" customHeight="1">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>592.7863833333333</v>
+        <v>592.7864</v>
       </c>
     </row>
     <row r="28" ht="14" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>593.3378666666666</v>
+        <v>593.3379</v>
       </c>
     </row>
     <row r="29" ht="14" customHeight="1">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>596.6757666666666</v>
+        <v>596.6758</v>
       </c>
     </row>
     <row r="30" ht="14" customHeight="1">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>597.78025</v>
+        <v>597.7802</v>
       </c>
     </row>
     <row r="31" ht="14" customHeight="1">
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>595.1624999999999</v>
+        <v>595.1625</v>
       </c>
     </row>
     <row r="32" ht="14" customHeight="1">
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>589.4851833333333</v>
+        <v>589.4852</v>
       </c>
     </row>
     <row r="34" ht="14" customHeight="1">
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>578.4554499999999</v>
+        <v>578.4554000000001</v>
       </c>
     </row>
     <row r="35" ht="14" customHeight="1">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>1383.659783333333</v>
+        <v>1383.6598</v>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1">
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>591.1401999999999</v>
+        <v>591.1402</v>
       </c>
     </row>
     <row r="37" ht="14" customHeight="1">
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="B68" s="7" t="n">
-        <v>575.1709166666666</v>
+        <v>575.1709</v>
       </c>
     </row>
     <row r="69" ht="14" customHeight="1">
@@ -1164,7 +1164,7 @@
         </is>
       </c>
       <c r="B71" s="7" t="n">
-        <v>179.2771713991827</v>
+        <v>179.2772</v>
       </c>
     </row>
     <row r="72" ht="14" customHeight="1">
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="B72" s="7" t="n">
-        <v>520.1245166666665</v>
+        <v>520.1245</v>
       </c>
     </row>
     <row r="73" ht="14" customHeight="1">
@@ -1184,7 +1184,7 @@
         </is>
       </c>
       <c r="B73" s="7" t="n">
-        <v>486.4028999999999</v>
+        <v>486.4029</v>
       </c>
     </row>
     <row r="74" ht="14" customHeight="1">
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="B74" s="7" t="n">
-        <v>480.4124499999999</v>
+        <v>480.4124</v>
       </c>
     </row>
     <row r="75" ht="14" customHeight="1">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B76" s="7" t="n">
-        <v>488.6069666666666</v>
+        <v>488.607</v>
       </c>
     </row>
     <row r="77" ht="14" customHeight="1">
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="B77" s="7" t="n">
-        <v>498.2707333333333</v>
+        <v>498.2707</v>
       </c>
     </row>
     <row r="78" ht="14" customHeight="1">
@@ -1364,7 +1364,7 @@
         </is>
       </c>
       <c r="B91" s="7" t="n">
-        <v>112.0898666666667</v>
+        <v>112.0899</v>
       </c>
     </row>
     <row r="92" ht="14" customHeight="1">
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="B92" s="7" t="n">
-        <v>266.7326936213991</v>
+        <v>266.7327</v>
       </c>
     </row>
     <row r="93" ht="14" customHeight="1">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B93" s="7" t="n">
-        <v>197.5235166666666</v>
+        <v>197.5235</v>
       </c>
     </row>
     <row r="94" ht="14" customHeight="1">
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B94" s="7" t="n">
-        <v>244.8140333333332</v>
+        <v>244.814</v>
       </c>
     </row>
     <row r="95" ht="14" customHeight="1">
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="B95" s="7" t="n">
-        <v>295.5346166666667</v>
+        <v>295.5346</v>
       </c>
     </row>
     <row r="96" ht="14" customHeight="1">
@@ -1424,7 +1424,7 @@
         </is>
       </c>
       <c r="B97" s="7" t="n">
-        <v>394.9314833333333</v>
+        <v>394.9315</v>
       </c>
     </row>
     <row r="98" ht="14" customHeight="1">
@@ -1434,7 +1434,7 @@
         </is>
       </c>
       <c r="B98" s="7" t="n">
-        <v>445.43165</v>
+        <v>445.4317</v>
       </c>
     </row>
     <row r="99" ht="14" customHeight="1">
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="B99" s="7" t="n">
-        <v>495.6965833333333</v>
+        <v>495.6966</v>
       </c>
     </row>
     <row r="100" ht="14" customHeight="1">
@@ -1454,7 +1454,7 @@
         </is>
       </c>
       <c r="B100" s="7" t="n">
-        <v>547.11905</v>
+        <v>547.119</v>
       </c>
     </row>
     <row r="101" ht="14" customHeight="1">
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="B101" s="7" t="n">
-        <v>599.9854333333333</v>
+        <v>599.9854</v>
       </c>
     </row>
     <row r="102" ht="14" customHeight="1">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="B102" s="7" t="n">
-        <v>635.4297499999999</v>
+        <v>635.4297</v>
       </c>
     </row>
     <row r="103" ht="14" customHeight="1">
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="B103" s="7" t="n">
-        <v>660.8306833333334</v>
+        <v>660.8307</v>
       </c>
     </row>
     <row r="104" ht="14" customHeight="1">
@@ -1494,7 +1494,7 @@
         </is>
       </c>
       <c r="B104" s="7" t="n">
-        <v>702.0369333333333</v>
+        <v>702.0368999999999</v>
       </c>
     </row>
     <row r="105" ht="14" customHeight="1">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="B105" s="7" t="n">
-        <v>738.0657833333332</v>
+        <v>738.0658</v>
       </c>
     </row>
     <row r="106" ht="14" customHeight="1">
@@ -1514,7 +1514,7 @@
         </is>
       </c>
       <c r="B106" s="7" t="n">
-        <v>775.9447166666666</v>
+        <v>775.9447</v>
       </c>
     </row>
     <row r="107" ht="14" customHeight="1">
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="B107" s="7" t="n">
-        <v>826.0832499999999</v>
+        <v>826.0832</v>
       </c>
     </row>
     <row r="108" ht="14" customHeight="1">
@@ -1534,7 +1534,7 @@
         </is>
       </c>
       <c r="B108" s="7" t="n">
-        <v>762.4227999999999</v>
+        <v>762.4228000000001</v>
       </c>
     </row>
     <row r="109" ht="14" customHeight="1">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="B109" s="7" t="n">
-        <v>636.9826166666667</v>
+        <v>636.9826</v>
       </c>
     </row>
     <row r="110" ht="14" customHeight="1">
@@ -1554,7 +1554,7 @@
         </is>
       </c>
       <c r="B110" s="7" t="n">
-        <v>531.8940499999999</v>
+        <v>531.894</v>
       </c>
     </row>
     <row r="111" ht="14" customHeight="1">
@@ -1564,7 +1564,7 @@
         </is>
       </c>
       <c r="B111" s="7" t="n">
-        <v>678.8305333333333</v>
+        <v>678.8305</v>
       </c>
     </row>
     <row r="112" ht="14" customHeight="1">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="B112" s="7" t="n">
-        <v>686.2684999999999</v>
+        <v>686.2685</v>
       </c>
     </row>
     <row r="113" ht="14" customHeight="1">
@@ -1584,7 +1584,7 @@
         </is>
       </c>
       <c r="B113" s="7" t="n">
-        <v>696.5043833333332</v>
+        <v>696.5044</v>
       </c>
     </row>
     <row r="114" ht="14" customHeight="1">
@@ -1714,7 +1714,7 @@
         </is>
       </c>
       <c r="B126" s="7" t="n">
-        <v>715.8689166666666</v>
+        <v>715.8689000000001</v>
       </c>
     </row>
     <row r="127" ht="14" customHeight="1">
@@ -1724,7 +1724,7 @@
         </is>
       </c>
       <c r="B127" s="7" t="n">
-        <v>717.0051166666667</v>
+        <v>717.0051</v>
       </c>
     </row>
     <row r="128" ht="14" customHeight="1">
@@ -1744,7 +1744,7 @@
         </is>
       </c>
       <c r="B129" s="7" t="n">
-        <v>717.0548666666666</v>
+        <v>717.0549</v>
       </c>
     </row>
     <row r="130" ht="14" customHeight="1">
@@ -1754,7 +1754,7 @@
         </is>
       </c>
       <c r="B130" s="7" t="n">
-        <v>720.4459666666667</v>
+        <v>720.446</v>
       </c>
     </row>
     <row r="131" ht="14" customHeight="1">
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="B131" s="7" t="n">
-        <v>738.1347166666666</v>
+        <v>738.1347</v>
       </c>
     </row>
     <row r="132" ht="14" customHeight="1">
@@ -1774,7 +1774,7 @@
         </is>
       </c>
       <c r="B132" s="7" t="n">
-        <v>671.6935666666666</v>
+        <v>671.6935999999999</v>
       </c>
     </row>
     <row r="133" ht="14" customHeight="1">
@@ -1784,7 +1784,7 @@
         </is>
       </c>
       <c r="B133" s="7" t="n">
-        <v>1393.790316666667</v>
+        <v>1393.7903</v>
       </c>
     </row>
     <row r="134" ht="14" customHeight="1">
@@ -1804,7 +1804,7 @@
         </is>
       </c>
       <c r="B135" s="7" t="n">
-        <v>568.8260499999999</v>
+        <v>568.826</v>
       </c>
     </row>
     <row r="136" ht="14" customHeight="1">
@@ -1814,7 +1814,7 @@
         </is>
       </c>
       <c r="B136" s="7" t="n">
-        <v>1396.98855</v>
+        <v>1396.9886</v>
       </c>
     </row>
     <row r="137" ht="14" customHeight="1">
@@ -1824,7 +1824,7 @@
         </is>
       </c>
       <c r="B137" s="7" t="n">
-        <v>1397.759866666667</v>
+        <v>1397.7599</v>
       </c>
     </row>
     <row r="138" ht="14" customHeight="1">
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="B138" s="7" t="n">
-        <v>566.7474333333332</v>
+        <v>566.7474</v>
       </c>
     </row>
     <row r="139" ht="14" customHeight="1">
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="B139" s="7" t="n">
-        <v>1399.873766666667</v>
+        <v>1399.8738</v>
       </c>
     </row>
     <row r="140" ht="14" customHeight="1">
@@ -1854,7 +1854,7 @@
         </is>
       </c>
       <c r="B140" s="7" t="n">
-        <v>567.83015</v>
+        <v>567.8302</v>
       </c>
     </row>
     <row r="141" ht="14" customHeight="1">
@@ -1864,7 +1864,7 @@
         </is>
       </c>
       <c r="B141" s="7" t="n">
-        <v>569.3586333333333</v>
+        <v>569.3586</v>
       </c>
     </row>
     <row r="142" ht="14" customHeight="1">
@@ -1874,7 +1874,7 @@
         </is>
       </c>
       <c r="B142" s="7" t="n">
-        <v>1403.663516666667</v>
+        <v>1403.6635</v>
       </c>
     </row>
     <row r="143" ht="14" customHeight="1">
@@ -1884,7 +1884,7 @@
         </is>
       </c>
       <c r="B143" s="7" t="n">
-        <v>904.9487166666668</v>
+        <v>904.9487</v>
       </c>
     </row>
     <row r="144" ht="14" customHeight="1">
@@ -1894,7 +1894,7 @@
         </is>
       </c>
       <c r="B144" s="7" t="n">
-        <v>573.1768333333333</v>
+        <v>573.1768</v>
       </c>
     </row>
     <row r="145" ht="14" customHeight="1">
@@ -1904,7 +1904,7 @@
         </is>
       </c>
       <c r="B145" s="7" t="n">
-        <v>574.1209833333332</v>
+        <v>574.121</v>
       </c>
     </row>
   </sheetData>
@@ -1919,7 +1919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14" customHeight="1"/>
   <cols>
     <col width="11.6328125" customWidth="1" style="4" min="1" max="3"/>
@@ -1970,6 +1970,9 @@
           <t>0:00</t>
         </is>
       </c>
+      <c r="E2" t="n">
+        <v>6000</v>
+      </c>
     </row>
     <row r="3" ht="14" customFormat="1" customHeight="1" s="5">
       <c r="A3" s="5" t="inlineStr">
@@ -1978,7 +1981,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>833.3333333333333</v>
+        <v>833.3333</v>
       </c>
       <c r="C3" t="n">
         <v>6365.8412</v>
@@ -1988,6 +1991,9 @@
           <t>24:00</t>
         </is>
       </c>
+      <c r="E3" t="n">
+        <v>6000</v>
+      </c>
     </row>
     <row r="4" ht="14" customFormat="1" customHeight="1" s="5">
       <c r="A4" s="5" t="inlineStr">
@@ -1996,10 +2002,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4787.964288065848</v>
+        <v>4787.9643</v>
       </c>
       <c r="C4" t="n">
-        <v>1702.996983333333</v>
+        <v>1702.997</v>
       </c>
     </row>
     <row r="5" ht="14" customFormat="1" customHeight="1" s="5">
@@ -2009,10 +2015,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5286.035176954732</v>
+        <v>5286.0352</v>
       </c>
       <c r="C5" t="n">
-        <v>91.10138333333346</v>
+        <v>91.1014</v>
       </c>
     </row>
     <row r="6" ht="14" customFormat="1" customHeight="1" s="5">
@@ -2025,7 +2031,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>5780.131883333333</v>
+        <v>5780.1319</v>
       </c>
     </row>
     <row r="7" ht="14" customFormat="1" customHeight="1" s="5">
@@ -2035,18 +2041,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5333.333333333333</v>
+        <v>5333.3333</v>
       </c>
       <c r="C7" t="n">
-        <v>2859.868116666667</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" t="n">
-        <v>6000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>6000</v>
+        <v>2859.8681</v>
       </c>
     </row>
   </sheetData>

</xml_diff>